<commit_message>
Updated data path and simulations
</commit_message>
<xml_diff>
--- a/MicroInstructions.xlsx
+++ b/MicroInstructions.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Raven\Documents\GitHub\Computer-Design-Final-Project\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C552516F-B6BB-44ED-B4E7-A967E4D343CC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{122F1425-A4C5-490A-993C-EF550E183C27}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-105" yWindow="0" windowWidth="19410" windowHeight="20985" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="84" uniqueCount="65">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="85" uniqueCount="66">
   <si>
     <t>Address</t>
   </si>
@@ -231,6 +231,9 @@
   </si>
   <si>
     <t>MemDump</t>
+  </si>
+  <si>
+    <t>Control bus for data path</t>
   </si>
 </sst>
 </file>
@@ -252,12 +255,18 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="2">
+  <fills count="3">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFFF00"/>
+        <bgColor indexed="64"/>
+      </patternFill>
     </fill>
   </fills>
   <borders count="1">
@@ -272,12 +281,21 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
@@ -560,7 +578,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A2:Q36"/>
+  <dimension ref="A1:Q36"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="9.28515625" style="1" bestFit="1" customWidth="1"/>
@@ -583,10 +601,34 @@
     <col min="18" max="16384" width="9.140625" style="1"/>
   </cols>
   <sheetData>
+    <row r="1" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="G1" s="3" t="s">
+        <v>65</v>
+      </c>
+      <c r="H1" s="3"/>
+      <c r="I1" s="3"/>
+      <c r="J1" s="3"/>
+      <c r="K1" s="3"/>
+      <c r="L1" s="3"/>
+      <c r="M1" s="3"/>
+      <c r="N1" s="3"/>
+      <c r="O1" s="3"/>
+      <c r="P1" s="3"/>
+    </row>
     <row r="2" spans="1:17" x14ac:dyDescent="0.25">
       <c r="C2" s="1" t="s">
         <v>33</v>
       </c>
+      <c r="G2" s="5"/>
+      <c r="H2" s="5"/>
+      <c r="I2" s="5"/>
+      <c r="J2" s="5"/>
+      <c r="K2" s="5"/>
+      <c r="L2" s="5"/>
+      <c r="M2" s="5"/>
+      <c r="N2" s="5"/>
+      <c r="O2" s="5"/>
+      <c r="P2" s="5"/>
     </row>
     <row r="3" spans="1:17" x14ac:dyDescent="0.25">
       <c r="B3" s="1" t="s">
@@ -604,34 +646,34 @@
       <c r="F3" s="1" t="s">
         <v>35</v>
       </c>
-      <c r="G3" s="1" t="s">
+      <c r="G3" s="4" t="s">
         <v>36</v>
       </c>
-      <c r="H3" s="1" t="s">
+      <c r="H3" s="4" t="s">
         <v>37</v>
       </c>
-      <c r="I3" s="1" t="s">
+      <c r="I3" s="4" t="s">
         <v>38</v>
       </c>
-      <c r="J3" s="1" t="s">
+      <c r="J3" s="4" t="s">
         <v>39</v>
       </c>
-      <c r="K3" s="1" t="s">
+      <c r="K3" s="4" t="s">
         <v>40</v>
       </c>
-      <c r="L3" s="1" t="s">
+      <c r="L3" s="4" t="s">
         <v>41</v>
       </c>
-      <c r="M3" s="1" t="s">
+      <c r="M3" s="4" t="s">
         <v>42</v>
       </c>
-      <c r="N3" s="1" t="s">
+      <c r="N3" s="4" t="s">
         <v>43</v>
       </c>
-      <c r="O3" s="1" t="s">
+      <c r="O3" s="4" t="s">
         <v>44</v>
       </c>
-      <c r="P3" s="1" t="s">
+      <c r="P3" s="4" t="s">
         <v>45</v>
       </c>
       <c r="Q3" s="1" t="s">
@@ -1398,6 +1440,9 @@
       <c r="B36" s="2"/>
     </row>
   </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="G1:P1"/>
+  </mergeCells>
   <phoneticPr fontId="1" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" r:id="rId1"/>

</xml_diff>

<commit_message>
Added support for JEQ via Z
</commit_message>
<xml_diff>
--- a/MicroInstructions.xlsx
+++ b/MicroInstructions.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="11003"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="29929"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/bradykirchberg/Documents/GitHub/Computer-Design-Final-Project/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Raven\Documents\GitHub\Computer-Design-Final-Project\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1DDFE76C-4201-9D48-B5F3-DB5D9B93DF6A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{35CAA844-6128-4F2F-92A4-34B9525DEAAC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="480" yWindow="660" windowWidth="27360" windowHeight="16040" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="10260" yWindow="6225" windowWidth="26730" windowHeight="14655" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="4-bit Addr" sheetId="2" r:id="rId1"/>
@@ -337,7 +337,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="3">
+  <borders count="6">
     <border>
       <left/>
       <right/>
@@ -367,11 +367,48 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right/>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="15">
+  <cellXfs count="20">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -391,9 +428,6 @@
     <xf numFmtId="3" fontId="1" fillId="3" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="3" fontId="1" fillId="2" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
     <xf numFmtId="49" fontId="1" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -405,6 +439,22 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="3" fontId="1" fillId="2" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="3" fontId="1" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="3" fontId="1" fillId="2" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="3" fontId="1" fillId="2" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="3" fontId="1" fillId="2" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="3" fontId="1" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -711,56 +761,56 @@
     <outlinePr summaryBelow="0"/>
   </sheetPr>
   <dimension ref="A1:S20"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr defaultColWidth="8.85546875" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="9.33203125" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="8.1640625" style="1" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="12.5" style="1" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="13.5" style="2" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="10.83203125" style="2" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="10.5" style="2" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="9.28515625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="8.140625" style="1" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="12.42578125" style="1" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="13.42578125" style="2" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="10.85546875" style="2" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="10.42578125" style="2" bestFit="1" customWidth="1"/>
     <col min="7" max="7" width="10" style="2" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="8.6640625" style="2" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="4.6640625" style="2" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="8.7109375" style="2" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="4.7109375" style="2" bestFit="1" customWidth="1"/>
     <col min="10" max="10" width="5" style="2" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="5.83203125" style="2" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="6.5" style="2" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="5.1640625" style="2" bestFit="1" customWidth="1"/>
-    <col min="14" max="14" width="6.5" style="2" bestFit="1" customWidth="1"/>
-    <col min="15" max="15" width="7.1640625" style="2" bestFit="1" customWidth="1"/>
-    <col min="16" max="16" width="5.1640625" style="2" bestFit="1" customWidth="1"/>
-    <col min="17" max="17" width="5.83203125" style="2" bestFit="1" customWidth="1"/>
-    <col min="18" max="18" width="4.5" style="2" bestFit="1" customWidth="1"/>
-    <col min="19" max="19" width="12.83203125" style="3" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="5.85546875" style="2" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="6.42578125" style="2" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="5.140625" style="2" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="6.42578125" style="2" bestFit="1" customWidth="1"/>
+    <col min="15" max="15" width="7.140625" style="2" bestFit="1" customWidth="1"/>
+    <col min="16" max="16" width="5.140625" style="2" bestFit="1" customWidth="1"/>
+    <col min="17" max="17" width="5.85546875" style="2" bestFit="1" customWidth="1"/>
+    <col min="18" max="18" width="4.42578125" style="2" bestFit="1" customWidth="1"/>
+    <col min="19" max="19" width="12.85546875" style="3" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:19" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A1" s="11"/>
-      <c r="B1" s="12"/>
-      <c r="C1" s="12"/>
+    <row r="1" spans="1:19" ht="17.25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A1" s="10"/>
+      <c r="B1" s="11"/>
+      <c r="C1" s="11"/>
       <c r="D1" s="6"/>
-      <c r="E1" s="5" t="s">
-        <v>0</v>
-      </c>
-      <c r="F1" s="5"/>
-      <c r="G1" s="5"/>
-      <c r="H1" s="5"/>
-      <c r="I1" s="5"/>
-      <c r="J1" s="5"/>
-      <c r="K1" s="5"/>
-      <c r="L1" s="5"/>
-      <c r="M1" s="5"/>
-      <c r="N1" s="5"/>
-      <c r="O1" s="5"/>
-      <c r="P1" s="5"/>
-      <c r="Q1" s="5"/>
-      <c r="R1" s="5"/>
-      <c r="S1" s="13"/>
-    </row>
-    <row r="2" spans="1:19" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A2" s="11"/>
-      <c r="B2" s="12"/>
-      <c r="C2" s="12" t="s">
+      <c r="E1" s="19"/>
+      <c r="F1" s="19"/>
+      <c r="G1" s="19"/>
+      <c r="H1" s="16" t="s">
+        <v>0</v>
+      </c>
+      <c r="I1" s="17"/>
+      <c r="J1" s="17"/>
+      <c r="K1" s="17"/>
+      <c r="L1" s="17"/>
+      <c r="M1" s="17"/>
+      <c r="N1" s="17"/>
+      <c r="O1" s="17"/>
+      <c r="P1" s="17"/>
+      <c r="Q1" s="17"/>
+      <c r="R1" s="18"/>
+      <c r="S1" s="12"/>
+    </row>
+    <row r="2" spans="1:19" ht="17.25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A2" s="10"/>
+      <c r="B2" s="11"/>
+      <c r="C2" s="11" t="s">
         <v>1</v>
       </c>
       <c r="D2" s="7" t="s">
@@ -780,71 +830,71 @@
       <c r="P2" s="7"/>
       <c r="Q2" s="7"/>
       <c r="R2" s="7"/>
-      <c r="S2" s="13"/>
-    </row>
-    <row r="3" spans="1:19" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A3" s="11"/>
-      <c r="B3" s="10" t="s">
+      <c r="S2" s="12"/>
+    </row>
+    <row r="3" spans="1:19" ht="17.25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A3" s="10"/>
+      <c r="B3" s="9" t="s">
         <v>3</v>
       </c>
-      <c r="C3" s="12"/>
+      <c r="C3" s="11"/>
       <c r="D3" s="7" t="s">
         <v>4</v>
       </c>
-      <c r="E3" s="8" t="s">
+      <c r="E3" s="15" t="s">
         <v>5</v>
       </c>
-      <c r="F3" s="8" t="s">
+      <c r="F3" s="15" t="s">
         <v>6</v>
       </c>
-      <c r="G3" s="8" t="s">
+      <c r="G3" s="15" t="s">
         <v>7</v>
       </c>
-      <c r="H3" s="9" t="s">
+      <c r="H3" s="5" t="s">
         <v>8</v>
       </c>
-      <c r="I3" s="9" t="s">
+      <c r="I3" s="5" t="s">
         <v>9</v>
       </c>
-      <c r="J3" s="9" t="s">
+      <c r="J3" s="5" t="s">
         <v>10</v>
       </c>
-      <c r="K3" s="9" t="s">
+      <c r="K3" s="5" t="s">
         <v>11</v>
       </c>
-      <c r="L3" s="9" t="s">
+      <c r="L3" s="5" t="s">
         <v>12</v>
       </c>
-      <c r="M3" s="9" t="s">
+      <c r="M3" s="5" t="s">
         <v>13</v>
       </c>
-      <c r="N3" s="9" t="s">
+      <c r="N3" s="5" t="s">
         <v>14</v>
       </c>
-      <c r="O3" s="9" t="s">
+      <c r="O3" s="5" t="s">
         <v>15</v>
       </c>
-      <c r="P3" s="9" t="s">
+      <c r="P3" s="5" t="s">
         <v>16</v>
       </c>
-      <c r="Q3" s="9" t="s">
+      <c r="Q3" s="5" t="s">
         <v>91</v>
       </c>
-      <c r="R3" s="9" t="s">
+      <c r="R3" s="5" t="s">
         <v>17</v>
       </c>
-      <c r="S3" s="10" t="s">
+      <c r="S3" s="9" t="s">
         <v>18</v>
       </c>
     </row>
-    <row r="4" spans="1:19" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A4" s="14" t="s">
+    <row r="4" spans="1:19" ht="17.25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A4" s="13" t="s">
         <v>19</v>
       </c>
-      <c r="B4" s="10" t="s">
+      <c r="B4" s="9" t="s">
         <v>74</v>
       </c>
-      <c r="C4" s="12"/>
+      <c r="C4" s="11"/>
       <c r="D4" s="7">
         <v>0</v>
       </c>
@@ -878,7 +928,7 @@
       <c r="N4" s="7">
         <v>0</v>
       </c>
-      <c r="O4" s="10" t="s">
+      <c r="O4" s="9" t="s">
         <v>21</v>
       </c>
       <c r="P4" s="7">
@@ -890,18 +940,18 @@
       <c r="R4" s="7">
         <v>0</v>
       </c>
-      <c r="S4" s="10" t="s">
+      <c r="S4" s="9" t="s">
         <v>75</v>
       </c>
     </row>
-    <row r="5" spans="1:19" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A5" s="14" t="s">
+    <row r="5" spans="1:19" ht="17.25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A5" s="13" t="s">
         <v>23</v>
       </c>
-      <c r="B5" s="10" t="s">
+      <c r="B5" s="9" t="s">
         <v>75</v>
       </c>
-      <c r="C5" s="12"/>
+      <c r="C5" s="11"/>
       <c r="D5" s="7">
         <v>0</v>
       </c>
@@ -935,7 +985,7 @@
       <c r="N5" s="7">
         <v>0</v>
       </c>
-      <c r="O5" s="10" t="s">
+      <c r="O5" s="9" t="s">
         <v>21</v>
       </c>
       <c r="P5" s="7">
@@ -947,18 +997,18 @@
       <c r="R5" s="7">
         <v>0</v>
       </c>
-      <c r="S5" s="10" t="s">
+      <c r="S5" s="9" t="s">
         <v>76</v>
       </c>
     </row>
-    <row r="6" spans="1:19" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A6" s="14" t="s">
+    <row r="6" spans="1:19" ht="17.25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A6" s="13" t="s">
         <v>25</v>
       </c>
-      <c r="B6" s="10" t="s">
+      <c r="B6" s="9" t="s">
         <v>76</v>
       </c>
-      <c r="C6" s="12"/>
+      <c r="C6" s="11"/>
       <c r="D6" s="7">
         <v>1</v>
       </c>
@@ -992,7 +1042,7 @@
       <c r="N6" s="7">
         <v>1</v>
       </c>
-      <c r="O6" s="10" t="s">
+      <c r="O6" s="9" t="s">
         <v>21</v>
       </c>
       <c r="P6" s="7">
@@ -1004,18 +1054,18 @@
       <c r="R6" s="7">
         <v>1</v>
       </c>
-      <c r="S6" s="10" t="s">
+      <c r="S6" s="9" t="s">
         <v>90</v>
       </c>
     </row>
-    <row r="7" spans="1:19" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A7" s="14" t="s">
+    <row r="7" spans="1:19" ht="17.25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A7" s="13" t="s">
         <v>55</v>
       </c>
-      <c r="B7" s="10" t="s">
+      <c r="B7" s="9" t="s">
         <v>77</v>
       </c>
-      <c r="C7" s="12"/>
+      <c r="C7" s="11"/>
       <c r="D7" s="7">
         <v>0</v>
       </c>
@@ -1049,7 +1099,7 @@
       <c r="N7" s="7">
         <v>1</v>
       </c>
-      <c r="O7" s="10" t="s">
+      <c r="O7" s="9" t="s">
         <v>56</v>
       </c>
       <c r="P7" s="7">
@@ -1061,18 +1111,18 @@
       <c r="R7" s="7">
         <v>0</v>
       </c>
-      <c r="S7" s="10" t="s">
+      <c r="S7" s="9" t="s">
         <v>74</v>
       </c>
     </row>
-    <row r="8" spans="1:19" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A8" s="14" t="s">
+    <row r="8" spans="1:19" ht="17.25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A8" s="13" t="s">
         <v>60</v>
       </c>
-      <c r="B8" s="10" t="s">
+      <c r="B8" s="9" t="s">
         <v>78</v>
       </c>
-      <c r="C8" s="12"/>
+      <c r="C8" s="11"/>
       <c r="D8" s="7">
         <v>0</v>
       </c>
@@ -1106,7 +1156,7 @@
       <c r="N8" s="7">
         <v>1</v>
       </c>
-      <c r="O8" s="10" t="s">
+      <c r="O8" s="9" t="s">
         <v>61</v>
       </c>
       <c r="P8" s="7">
@@ -1118,16 +1168,16 @@
       <c r="R8" s="7">
         <v>0</v>
       </c>
-      <c r="S8" s="10" t="s">
+      <c r="S8" s="9" t="s">
         <v>74</v>
       </c>
     </row>
-    <row r="9" spans="1:19" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A9" s="11"/>
-      <c r="B9" s="10" t="s">
+    <row r="9" spans="1:19" ht="17.25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A9" s="10"/>
+      <c r="B9" s="9" t="s">
         <v>79</v>
       </c>
-      <c r="C9" s="12"/>
+      <c r="C9" s="11"/>
       <c r="D9" s="6"/>
       <c r="E9" s="6"/>
       <c r="F9" s="6"/>
@@ -1143,14 +1193,14 @@
       <c r="P9" s="6"/>
       <c r="Q9" s="6"/>
       <c r="R9" s="6"/>
-      <c r="S9" s="13"/>
-    </row>
-    <row r="10" spans="1:19" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A10" s="11"/>
-      <c r="B10" s="10" t="s">
+      <c r="S9" s="12"/>
+    </row>
+    <row r="10" spans="1:19" ht="17.25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A10" s="10"/>
+      <c r="B10" s="9" t="s">
         <v>80</v>
       </c>
-      <c r="C10" s="12"/>
+      <c r="C10" s="11"/>
       <c r="D10" s="6"/>
       <c r="E10" s="6"/>
       <c r="F10" s="6"/>
@@ -1166,14 +1216,14 @@
       <c r="P10" s="6"/>
       <c r="Q10" s="6"/>
       <c r="R10" s="6"/>
-      <c r="S10" s="13"/>
-    </row>
-    <row r="11" spans="1:19" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A11" s="11"/>
-      <c r="B11" s="10" t="s">
+      <c r="S10" s="12"/>
+    </row>
+    <row r="11" spans="1:19" ht="17.25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A11" s="10"/>
+      <c r="B11" s="9" t="s">
         <v>81</v>
       </c>
-      <c r="C11" s="12"/>
+      <c r="C11" s="11"/>
       <c r="D11" s="6"/>
       <c r="E11" s="6"/>
       <c r="F11" s="6"/>
@@ -1189,16 +1239,16 @@
       <c r="P11" s="6"/>
       <c r="Q11" s="6"/>
       <c r="R11" s="6"/>
-      <c r="S11" s="13"/>
-    </row>
-    <row r="12" spans="1:19" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A12" s="14" t="s">
+      <c r="S11" s="12"/>
+    </row>
+    <row r="12" spans="1:19" ht="17.25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A12" s="13" t="s">
         <v>40</v>
       </c>
-      <c r="B12" s="10" t="s">
+      <c r="B12" s="9" t="s">
         <v>82</v>
       </c>
-      <c r="C12" s="12" t="s">
+      <c r="C12" s="11" t="s">
         <v>67</v>
       </c>
       <c r="D12" s="7">
@@ -1234,7 +1284,7 @@
       <c r="N12" s="7">
         <v>0</v>
       </c>
-      <c r="O12" s="10" t="s">
+      <c r="O12" s="9" t="s">
         <v>21</v>
       </c>
       <c r="P12" s="7">
@@ -1246,18 +1296,18 @@
       <c r="R12" s="7">
         <v>0</v>
       </c>
-      <c r="S12" s="10" t="s">
+      <c r="S12" s="9" t="s">
         <v>74</v>
       </c>
     </row>
-    <row r="13" spans="1:19" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A13" s="14" t="s">
+    <row r="13" spans="1:19" ht="17.25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A13" s="13" t="s">
         <v>43</v>
       </c>
-      <c r="B13" s="10" t="s">
+      <c r="B13" s="9" t="s">
         <v>83</v>
       </c>
-      <c r="C13" s="12" t="s">
+      <c r="C13" s="11" t="s">
         <v>68</v>
       </c>
       <c r="D13" s="7">
@@ -1293,7 +1343,7 @@
       <c r="N13" s="7">
         <v>0</v>
       </c>
-      <c r="O13" s="10" t="s">
+      <c r="O13" s="9" t="s">
         <v>21</v>
       </c>
       <c r="P13" s="7">
@@ -1305,18 +1355,18 @@
       <c r="R13" s="7">
         <v>0</v>
       </c>
-      <c r="S13" s="10" t="s">
+      <c r="S13" s="9" t="s">
         <v>74</v>
       </c>
     </row>
-    <row r="14" spans="1:19" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A14" s="14" t="s">
+    <row r="14" spans="1:19" ht="17.25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A14" s="13" t="s">
         <v>46</v>
       </c>
-      <c r="B14" s="10" t="s">
+      <c r="B14" s="9" t="s">
         <v>84</v>
       </c>
-      <c r="C14" s="12" t="s">
+      <c r="C14" s="11" t="s">
         <v>69</v>
       </c>
       <c r="D14" s="7">
@@ -1352,7 +1402,7 @@
       <c r="N14" s="7">
         <v>1</v>
       </c>
-      <c r="O14" s="10" t="s">
+      <c r="O14" s="9" t="s">
         <v>21</v>
       </c>
       <c r="P14" s="7">
@@ -1364,18 +1414,18 @@
       <c r="R14" s="7">
         <v>0</v>
       </c>
-      <c r="S14" s="10" t="s">
+      <c r="S14" s="9" t="s">
         <v>74</v>
       </c>
     </row>
-    <row r="15" spans="1:19" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A15" s="14" t="s">
+    <row r="15" spans="1:19" ht="17.25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A15" s="13" t="s">
         <v>49</v>
       </c>
-      <c r="B15" s="10" t="s">
+      <c r="B15" s="9" t="s">
         <v>85</v>
       </c>
-      <c r="C15" s="12" t="s">
+      <c r="C15" s="11" t="s">
         <v>70</v>
       </c>
       <c r="D15" s="7">
@@ -1411,7 +1461,7 @@
       <c r="N15" s="7">
         <v>1</v>
       </c>
-      <c r="O15" s="10" t="s">
+      <c r="O15" s="9" t="s">
         <v>21</v>
       </c>
       <c r="P15" s="7">
@@ -1423,18 +1473,18 @@
       <c r="R15" s="7">
         <v>0</v>
       </c>
-      <c r="S15" s="10" t="s">
+      <c r="S15" s="9" t="s">
         <v>74</v>
       </c>
     </row>
-    <row r="16" spans="1:19" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A16" s="14" t="s">
+    <row r="16" spans="1:19" ht="17.25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A16" s="13" t="s">
         <v>52</v>
       </c>
-      <c r="B16" s="10" t="s">
+      <c r="B16" s="9" t="s">
         <v>86</v>
       </c>
-      <c r="C16" s="12" t="s">
+      <c r="C16" s="11" t="s">
         <v>71</v>
       </c>
       <c r="D16" s="7">
@@ -1470,7 +1520,7 @@
       <c r="N16" s="7">
         <v>0</v>
       </c>
-      <c r="O16" s="10" t="s">
+      <c r="O16" s="9" t="s">
         <v>21</v>
       </c>
       <c r="P16" s="7">
@@ -1482,18 +1532,18 @@
       <c r="R16" s="7">
         <v>0</v>
       </c>
-      <c r="S16" s="10" t="s">
+      <c r="S16" s="9" t="s">
         <v>77</v>
       </c>
     </row>
-    <row r="17" spans="1:19" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A17" s="14" t="s">
+    <row r="17" spans="1:19" ht="17.25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A17" s="13" t="s">
         <v>57</v>
       </c>
-      <c r="B17" s="10" t="s">
+      <c r="B17" s="9" t="s">
         <v>87</v>
       </c>
-      <c r="C17" s="12" t="s">
+      <c r="C17" s="11" t="s">
         <v>72</v>
       </c>
       <c r="D17" s="7">
@@ -1529,7 +1579,7 @@
       <c r="N17" s="7">
         <v>0</v>
       </c>
-      <c r="O17" s="10" t="s">
+      <c r="O17" s="9" t="s">
         <v>21</v>
       </c>
       <c r="P17" s="7">
@@ -1541,16 +1591,16 @@
       <c r="R17" s="7">
         <v>0</v>
       </c>
-      <c r="S17" s="10" t="s">
+      <c r="S17" s="9" t="s">
         <v>78</v>
       </c>
     </row>
-    <row r="18" spans="1:19" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A18" s="14"/>
-      <c r="B18" s="10" t="s">
+    <row r="18" spans="1:19" ht="17.25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A18" s="13"/>
+      <c r="B18" s="9" t="s">
         <v>88</v>
       </c>
-      <c r="C18" s="12"/>
+      <c r="C18" s="11"/>
       <c r="D18" s="7"/>
       <c r="E18" s="7"/>
       <c r="F18" s="7"/>
@@ -1562,20 +1612,20 @@
       <c r="L18" s="7"/>
       <c r="M18" s="7"/>
       <c r="N18" s="7"/>
-      <c r="O18" s="10"/>
+      <c r="O18" s="9"/>
       <c r="P18" s="7"/>
       <c r="Q18" s="7"/>
       <c r="R18" s="7"/>
-      <c r="S18" s="10"/>
-    </row>
-    <row r="19" spans="1:19" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A19" s="14" t="s">
+      <c r="S18" s="9"/>
+    </row>
+    <row r="19" spans="1:19" ht="17.25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A19" s="13" t="s">
         <v>64</v>
       </c>
-      <c r="B19" s="10" t="s">
+      <c r="B19" s="9" t="s">
         <v>89</v>
       </c>
-      <c r="C19" s="12" t="s">
+      <c r="C19" s="11" t="s">
         <v>73</v>
       </c>
       <c r="D19" s="7">
@@ -1621,16 +1671,16 @@
       <c r="R19" s="7">
         <v>0</v>
       </c>
-      <c r="S19" s="10" t="s">
+      <c r="S19" s="9" t="s">
         <v>90</v>
       </c>
     </row>
-    <row r="20" spans="1:19" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="20" spans="1:19" ht="17.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B20" s="4"/>
     </row>
   </sheetData>
   <mergeCells count="1">
-    <mergeCell ref="E1:R1"/>
+    <mergeCell ref="H1:R1"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -1642,54 +1692,54 @@
     <outlinePr summaryBelow="0"/>
   </sheetPr>
   <dimension ref="A1:R36"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr defaultColWidth="8.85546875" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="9.33203125" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="8.1640625" style="1" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="12.5" style="1" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="13.5" style="2" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="10.83203125" style="2" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="10.5" style="2" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="9.28515625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="8.140625" style="1" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="12.42578125" style="1" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="13.42578125" style="2" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="10.85546875" style="2" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="10.42578125" style="2" bestFit="1" customWidth="1"/>
     <col min="7" max="7" width="10" style="2" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="8.6640625" style="2" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="4.6640625" style="2" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="8.7109375" style="2" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="4.7109375" style="2" bestFit="1" customWidth="1"/>
     <col min="10" max="10" width="5" style="2" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="5.83203125" style="2" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="6.5" style="2" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="5.1640625" style="2" bestFit="1" customWidth="1"/>
-    <col min="14" max="14" width="6.5" style="2" bestFit="1" customWidth="1"/>
-    <col min="15" max="15" width="7.1640625" style="2" bestFit="1" customWidth="1"/>
-    <col min="16" max="16" width="5.1640625" style="2" bestFit="1" customWidth="1"/>
-    <col min="17" max="17" width="4.5" style="2" bestFit="1" customWidth="1"/>
-    <col min="18" max="18" width="12.83203125" style="3" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="5.85546875" style="2" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="6.42578125" style="2" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="5.140625" style="2" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="6.42578125" style="2" bestFit="1" customWidth="1"/>
+    <col min="15" max="15" width="7.140625" style="2" bestFit="1" customWidth="1"/>
+    <col min="16" max="16" width="5.140625" style="2" bestFit="1" customWidth="1"/>
+    <col min="17" max="17" width="4.42578125" style="2" bestFit="1" customWidth="1"/>
+    <col min="18" max="18" width="12.85546875" style="3" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:18" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A1" s="11"/>
-      <c r="B1" s="12"/>
-      <c r="C1" s="12"/>
+    <row r="1" spans="1:18" ht="17.25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A1" s="10"/>
+      <c r="B1" s="11"/>
+      <c r="C1" s="11"/>
       <c r="D1" s="6"/>
-      <c r="E1" s="5" t="s">
-        <v>0</v>
-      </c>
-      <c r="F1" s="5"/>
-      <c r="G1" s="5"/>
-      <c r="H1" s="5"/>
-      <c r="I1" s="5"/>
-      <c r="J1" s="5"/>
-      <c r="K1" s="5"/>
-      <c r="L1" s="5"/>
-      <c r="M1" s="5"/>
-      <c r="N1" s="5"/>
-      <c r="O1" s="5"/>
-      <c r="P1" s="5"/>
-      <c r="Q1" s="5"/>
-      <c r="R1" s="13"/>
-    </row>
-    <row r="2" spans="1:18" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A2" s="11"/>
-      <c r="B2" s="12"/>
-      <c r="C2" s="12" t="s">
+      <c r="E1" s="14" t="s">
+        <v>0</v>
+      </c>
+      <c r="F1" s="14"/>
+      <c r="G1" s="14"/>
+      <c r="H1" s="14"/>
+      <c r="I1" s="14"/>
+      <c r="J1" s="14"/>
+      <c r="K1" s="14"/>
+      <c r="L1" s="14"/>
+      <c r="M1" s="14"/>
+      <c r="N1" s="14"/>
+      <c r="O1" s="14"/>
+      <c r="P1" s="14"/>
+      <c r="Q1" s="14"/>
+      <c r="R1" s="12"/>
+    </row>
+    <row r="2" spans="1:18" ht="17.25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A2" s="10"/>
+      <c r="B2" s="11"/>
+      <c r="C2" s="11" t="s">
         <v>1</v>
       </c>
       <c r="D2" s="7" t="s">
@@ -1708,14 +1758,14 @@
       <c r="O2" s="7"/>
       <c r="P2" s="7"/>
       <c r="Q2" s="7"/>
-      <c r="R2" s="13"/>
-    </row>
-    <row r="3" spans="1:18" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A3" s="11"/>
-      <c r="B3" s="10" t="s">
+      <c r="R2" s="12"/>
+    </row>
+    <row r="3" spans="1:18" ht="17.25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A3" s="10"/>
+      <c r="B3" s="9" t="s">
         <v>3</v>
       </c>
-      <c r="C3" s="12"/>
+      <c r="C3" s="11"/>
       <c r="D3" s="7" t="s">
         <v>4</v>
       </c>
@@ -1728,48 +1778,48 @@
       <c r="G3" s="8" t="s">
         <v>7</v>
       </c>
-      <c r="H3" s="9" t="s">
+      <c r="H3" s="5" t="s">
         <v>8</v>
       </c>
-      <c r="I3" s="9" t="s">
+      <c r="I3" s="5" t="s">
         <v>9</v>
       </c>
-      <c r="J3" s="9" t="s">
+      <c r="J3" s="5" t="s">
         <v>10</v>
       </c>
-      <c r="K3" s="9" t="s">
+      <c r="K3" s="5" t="s">
         <v>11</v>
       </c>
-      <c r="L3" s="9" t="s">
+      <c r="L3" s="5" t="s">
         <v>12</v>
       </c>
-      <c r="M3" s="9" t="s">
+      <c r="M3" s="5" t="s">
         <v>13</v>
       </c>
-      <c r="N3" s="9" t="s">
+      <c r="N3" s="5" t="s">
         <v>14</v>
       </c>
-      <c r="O3" s="9" t="s">
+      <c r="O3" s="5" t="s">
         <v>15</v>
       </c>
-      <c r="P3" s="9" t="s">
+      <c r="P3" s="5" t="s">
         <v>16</v>
       </c>
-      <c r="Q3" s="9" t="s">
+      <c r="Q3" s="5" t="s">
         <v>17</v>
       </c>
-      <c r="R3" s="10" t="s">
+      <c r="R3" s="9" t="s">
         <v>18</v>
       </c>
     </row>
-    <row r="4" spans="1:18" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A4" s="14" t="s">
+    <row r="4" spans="1:18" ht="17.25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A4" s="13" t="s">
         <v>19</v>
       </c>
-      <c r="B4" s="10" t="s">
+      <c r="B4" s="9" t="s">
         <v>20</v>
       </c>
-      <c r="C4" s="12"/>
+      <c r="C4" s="11"/>
       <c r="D4" s="7">
         <v>0</v>
       </c>
@@ -1803,7 +1853,7 @@
       <c r="N4" s="7">
         <v>0</v>
       </c>
-      <c r="O4" s="10" t="s">
+      <c r="O4" s="9" t="s">
         <v>21</v>
       </c>
       <c r="P4" s="7">
@@ -1812,18 +1862,18 @@
       <c r="Q4" s="7">
         <v>0</v>
       </c>
-      <c r="R4" s="10" t="s">
+      <c r="R4" s="9" t="s">
         <v>22</v>
       </c>
     </row>
-    <row r="5" spans="1:18" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A5" s="14" t="s">
+    <row r="5" spans="1:18" ht="17.25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A5" s="13" t="s">
         <v>23</v>
       </c>
-      <c r="B5" s="10" t="s">
+      <c r="B5" s="9" t="s">
         <v>22</v>
       </c>
-      <c r="C5" s="12"/>
+      <c r="C5" s="11"/>
       <c r="D5" s="7">
         <v>0</v>
       </c>
@@ -1857,7 +1907,7 @@
       <c r="N5" s="7">
         <v>0</v>
       </c>
-      <c r="O5" s="10" t="s">
+      <c r="O5" s="9" t="s">
         <v>21</v>
       </c>
       <c r="P5" s="7">
@@ -1866,18 +1916,18 @@
       <c r="Q5" s="7">
         <v>0</v>
       </c>
-      <c r="R5" s="10" t="s">
+      <c r="R5" s="9" t="s">
         <v>24</v>
       </c>
     </row>
-    <row r="6" spans="1:18" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A6" s="14" t="s">
+    <row r="6" spans="1:18" ht="17.25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A6" s="13" t="s">
         <v>25</v>
       </c>
-      <c r="B6" s="10" t="s">
+      <c r="B6" s="9" t="s">
         <v>24</v>
       </c>
-      <c r="C6" s="12"/>
+      <c r="C6" s="11"/>
       <c r="D6" s="7">
         <v>1</v>
       </c>
@@ -1911,7 +1961,7 @@
       <c r="N6" s="7">
         <v>1</v>
       </c>
-      <c r="O6" s="10" t="s">
+      <c r="O6" s="9" t="s">
         <v>21</v>
       </c>
       <c r="P6" s="7">
@@ -1920,16 +1970,16 @@
       <c r="Q6" s="7">
         <v>1</v>
       </c>
-      <c r="R6" s="10" t="s">
+      <c r="R6" s="9" t="s">
         <v>26</v>
       </c>
     </row>
-    <row r="7" spans="1:18" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A7" s="11"/>
-      <c r="B7" s="10" t="s">
+    <row r="7" spans="1:18" ht="17.25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A7" s="10"/>
+      <c r="B7" s="9" t="s">
         <v>27</v>
       </c>
-      <c r="C7" s="12"/>
+      <c r="C7" s="11"/>
       <c r="D7" s="6"/>
       <c r="E7" s="6"/>
       <c r="F7" s="6"/>
@@ -1944,14 +1994,14 @@
       <c r="O7" s="7"/>
       <c r="P7" s="6"/>
       <c r="Q7" s="6"/>
-      <c r="R7" s="13"/>
-    </row>
-    <row r="8" spans="1:18" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A8" s="11"/>
-      <c r="B8" s="10" t="s">
+      <c r="R7" s="12"/>
+    </row>
+    <row r="8" spans="1:18" ht="17.25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A8" s="10"/>
+      <c r="B8" s="9" t="s">
         <v>28</v>
       </c>
-      <c r="C8" s="12"/>
+      <c r="C8" s="11"/>
       <c r="D8" s="6"/>
       <c r="E8" s="6"/>
       <c r="F8" s="6"/>
@@ -1966,14 +2016,14 @@
       <c r="O8" s="7"/>
       <c r="P8" s="6"/>
       <c r="Q8" s="6"/>
-      <c r="R8" s="13"/>
-    </row>
-    <row r="9" spans="1:18" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A9" s="11"/>
-      <c r="B9" s="10" t="s">
+      <c r="R8" s="12"/>
+    </row>
+    <row r="9" spans="1:18" ht="17.25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A9" s="10"/>
+      <c r="B9" s="9" t="s">
         <v>29</v>
       </c>
-      <c r="C9" s="12"/>
+      <c r="C9" s="11"/>
       <c r="D9" s="6"/>
       <c r="E9" s="6"/>
       <c r="F9" s="6"/>
@@ -1988,14 +2038,14 @@
       <c r="O9" s="7"/>
       <c r="P9" s="6"/>
       <c r="Q9" s="6"/>
-      <c r="R9" s="13"/>
-    </row>
-    <row r="10" spans="1:18" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A10" s="11"/>
-      <c r="B10" s="10" t="s">
+      <c r="R9" s="12"/>
+    </row>
+    <row r="10" spans="1:18" ht="17.25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A10" s="10"/>
+      <c r="B10" s="9" t="s">
         <v>30</v>
       </c>
-      <c r="C10" s="12"/>
+      <c r="C10" s="11"/>
       <c r="D10" s="6"/>
       <c r="E10" s="6"/>
       <c r="F10" s="6"/>
@@ -2010,14 +2060,14 @@
       <c r="O10" s="7"/>
       <c r="P10" s="6"/>
       <c r="Q10" s="6"/>
-      <c r="R10" s="13"/>
-    </row>
-    <row r="11" spans="1:18" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A11" s="11"/>
-      <c r="B11" s="10" t="s">
+      <c r="R10" s="12"/>
+    </row>
+    <row r="11" spans="1:18" ht="17.25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A11" s="10"/>
+      <c r="B11" s="9" t="s">
         <v>31</v>
       </c>
-      <c r="C11" s="12"/>
+      <c r="C11" s="11"/>
       <c r="D11" s="6"/>
       <c r="E11" s="6"/>
       <c r="F11" s="6"/>
@@ -2032,14 +2082,14 @@
       <c r="O11" s="7"/>
       <c r="P11" s="6"/>
       <c r="Q11" s="6"/>
-      <c r="R11" s="13"/>
-    </row>
-    <row r="12" spans="1:18" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A12" s="11"/>
-      <c r="B12" s="10" t="s">
+      <c r="R11" s="12"/>
+    </row>
+    <row r="12" spans="1:18" ht="17.25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A12" s="10"/>
+      <c r="B12" s="9" t="s">
         <v>32</v>
       </c>
-      <c r="C12" s="12"/>
+      <c r="C12" s="11"/>
       <c r="D12" s="6"/>
       <c r="E12" s="6"/>
       <c r="F12" s="6"/>
@@ -2054,14 +2104,14 @@
       <c r="O12" s="7"/>
       <c r="P12" s="6"/>
       <c r="Q12" s="6"/>
-      <c r="R12" s="13"/>
-    </row>
-    <row r="13" spans="1:18" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A13" s="11"/>
-      <c r="B13" s="10" t="s">
+      <c r="R12" s="12"/>
+    </row>
+    <row r="13" spans="1:18" ht="17.25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A13" s="10"/>
+      <c r="B13" s="9" t="s">
         <v>33</v>
       </c>
-      <c r="C13" s="12"/>
+      <c r="C13" s="11"/>
       <c r="D13" s="6"/>
       <c r="E13" s="6"/>
       <c r="F13" s="6"/>
@@ -2076,14 +2126,14 @@
       <c r="O13" s="7"/>
       <c r="P13" s="6"/>
       <c r="Q13" s="6"/>
-      <c r="R13" s="13"/>
-    </row>
-    <row r="14" spans="1:18" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A14" s="11"/>
-      <c r="B14" s="10" t="s">
+      <c r="R13" s="12"/>
+    </row>
+    <row r="14" spans="1:18" ht="17.25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A14" s="10"/>
+      <c r="B14" s="9" t="s">
         <v>34</v>
       </c>
-      <c r="C14" s="12"/>
+      <c r="C14" s="11"/>
       <c r="D14" s="6"/>
       <c r="E14" s="6"/>
       <c r="F14" s="6"/>
@@ -2098,14 +2148,14 @@
       <c r="O14" s="7"/>
       <c r="P14" s="6"/>
       <c r="Q14" s="6"/>
-      <c r="R14" s="13"/>
-    </row>
-    <row r="15" spans="1:18" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A15" s="11"/>
-      <c r="B15" s="10" t="s">
+      <c r="R14" s="12"/>
+    </row>
+    <row r="15" spans="1:18" ht="17.25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A15" s="10"/>
+      <c r="B15" s="9" t="s">
         <v>35</v>
       </c>
-      <c r="C15" s="12"/>
+      <c r="C15" s="11"/>
       <c r="D15" s="6"/>
       <c r="E15" s="6"/>
       <c r="F15" s="6"/>
@@ -2120,14 +2170,14 @@
       <c r="O15" s="7"/>
       <c r="P15" s="6"/>
       <c r="Q15" s="6"/>
-      <c r="R15" s="13"/>
-    </row>
-    <row r="16" spans="1:18" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A16" s="11"/>
-      <c r="B16" s="10" t="s">
+      <c r="R15" s="12"/>
+    </row>
+    <row r="16" spans="1:18" ht="17.25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A16" s="10"/>
+      <c r="B16" s="9" t="s">
         <v>36</v>
       </c>
-      <c r="C16" s="12"/>
+      <c r="C16" s="11"/>
       <c r="D16" s="6"/>
       <c r="E16" s="6"/>
       <c r="F16" s="6"/>
@@ -2142,14 +2192,14 @@
       <c r="O16" s="7"/>
       <c r="P16" s="6"/>
       <c r="Q16" s="6"/>
-      <c r="R16" s="13"/>
-    </row>
-    <row r="17" spans="1:18" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A17" s="11"/>
-      <c r="B17" s="10" t="s">
+      <c r="R16" s="12"/>
+    </row>
+    <row r="17" spans="1:18" ht="17.25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A17" s="10"/>
+      <c r="B17" s="9" t="s">
         <v>37</v>
       </c>
-      <c r="C17" s="12"/>
+      <c r="C17" s="11"/>
       <c r="D17" s="6"/>
       <c r="E17" s="6"/>
       <c r="F17" s="6"/>
@@ -2164,14 +2214,14 @@
       <c r="O17" s="7"/>
       <c r="P17" s="6"/>
       <c r="Q17" s="6"/>
-      <c r="R17" s="13"/>
-    </row>
-    <row r="18" spans="1:18" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A18" s="11"/>
-      <c r="B18" s="10" t="s">
+      <c r="R17" s="12"/>
+    </row>
+    <row r="18" spans="1:18" ht="17.25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A18" s="10"/>
+      <c r="B18" s="9" t="s">
         <v>38</v>
       </c>
-      <c r="C18" s="12"/>
+      <c r="C18" s="11"/>
       <c r="D18" s="6"/>
       <c r="E18" s="6"/>
       <c r="F18" s="6"/>
@@ -2186,14 +2236,14 @@
       <c r="O18" s="7"/>
       <c r="P18" s="6"/>
       <c r="Q18" s="6"/>
-      <c r="R18" s="13"/>
-    </row>
-    <row r="19" spans="1:18" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A19" s="11"/>
-      <c r="B19" s="10" t="s">
+      <c r="R18" s="12"/>
+    </row>
+    <row r="19" spans="1:18" ht="17.25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A19" s="10"/>
+      <c r="B19" s="9" t="s">
         <v>39</v>
       </c>
-      <c r="C19" s="12"/>
+      <c r="C19" s="11"/>
       <c r="D19" s="6"/>
       <c r="E19" s="6"/>
       <c r="F19" s="6"/>
@@ -2208,16 +2258,16 @@
       <c r="O19" s="7"/>
       <c r="P19" s="6"/>
       <c r="Q19" s="6"/>
-      <c r="R19" s="13"/>
-    </row>
-    <row r="20" spans="1:18" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A20" s="14" t="s">
+      <c r="R19" s="12"/>
+    </row>
+    <row r="20" spans="1:18" ht="17.25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A20" s="13" t="s">
         <v>40</v>
       </c>
-      <c r="B20" s="10" t="s">
+      <c r="B20" s="9" t="s">
         <v>41</v>
       </c>
-      <c r="C20" s="12" t="s">
+      <c r="C20" s="11" t="s">
         <v>67</v>
       </c>
       <c r="D20" s="7">
@@ -2253,7 +2303,7 @@
       <c r="N20" s="7">
         <v>0</v>
       </c>
-      <c r="O20" s="10" t="s">
+      <c r="O20" s="9" t="s">
         <v>21</v>
       </c>
       <c r="P20" s="7">
@@ -2262,16 +2312,16 @@
       <c r="Q20" s="7">
         <v>0</v>
       </c>
-      <c r="R20" s="10" t="s">
+      <c r="R20" s="9" t="s">
         <v>20</v>
       </c>
     </row>
-    <row r="21" spans="1:18" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A21" s="11"/>
-      <c r="B21" s="10" t="s">
+    <row r="21" spans="1:18" ht="17.25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A21" s="10"/>
+      <c r="B21" s="9" t="s">
         <v>42</v>
       </c>
-      <c r="C21" s="12"/>
+      <c r="C21" s="11"/>
       <c r="D21" s="6"/>
       <c r="E21" s="6"/>
       <c r="F21" s="6"/>
@@ -2286,16 +2336,16 @@
       <c r="O21" s="7"/>
       <c r="P21" s="6"/>
       <c r="Q21" s="6"/>
-      <c r="R21" s="13"/>
-    </row>
-    <row r="22" spans="1:18" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A22" s="14" t="s">
+      <c r="R21" s="12"/>
+    </row>
+    <row r="22" spans="1:18" ht="17.25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A22" s="13" t="s">
         <v>43</v>
       </c>
-      <c r="B22" s="10" t="s">
+      <c r="B22" s="9" t="s">
         <v>44</v>
       </c>
-      <c r="C22" s="12" t="s">
+      <c r="C22" s="11" t="s">
         <v>68</v>
       </c>
       <c r="D22" s="7">
@@ -2331,7 +2381,7 @@
       <c r="N22" s="7">
         <v>0</v>
       </c>
-      <c r="O22" s="10" t="s">
+      <c r="O22" s="9" t="s">
         <v>21</v>
       </c>
       <c r="P22" s="7">
@@ -2340,16 +2390,16 @@
       <c r="Q22" s="7">
         <v>0</v>
       </c>
-      <c r="R22" s="10" t="s">
+      <c r="R22" s="9" t="s">
         <v>20</v>
       </c>
     </row>
-    <row r="23" spans="1:18" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A23" s="11"/>
-      <c r="B23" s="10" t="s">
+    <row r="23" spans="1:18" ht="17.25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A23" s="10"/>
+      <c r="B23" s="9" t="s">
         <v>45</v>
       </c>
-      <c r="C23" s="12"/>
+      <c r="C23" s="11"/>
       <c r="D23" s="6"/>
       <c r="E23" s="6"/>
       <c r="F23" s="6"/>
@@ -2364,16 +2414,16 @@
       <c r="O23" s="7"/>
       <c r="P23" s="6"/>
       <c r="Q23" s="6"/>
-      <c r="R23" s="13"/>
-    </row>
-    <row r="24" spans="1:18" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A24" s="14" t="s">
+      <c r="R23" s="12"/>
+    </row>
+    <row r="24" spans="1:18" ht="17.25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A24" s="13" t="s">
         <v>46</v>
       </c>
-      <c r="B24" s="10" t="s">
+      <c r="B24" s="9" t="s">
         <v>47</v>
       </c>
-      <c r="C24" s="12" t="s">
+      <c r="C24" s="11" t="s">
         <v>69</v>
       </c>
       <c r="D24" s="7">
@@ -2409,7 +2459,7 @@
       <c r="N24" s="7">
         <v>1</v>
       </c>
-      <c r="O24" s="10" t="s">
+      <c r="O24" s="9" t="s">
         <v>21</v>
       </c>
       <c r="P24" s="7">
@@ -2418,16 +2468,16 @@
       <c r="Q24" s="7">
         <v>0</v>
       </c>
-      <c r="R24" s="10" t="s">
+      <c r="R24" s="9" t="s">
         <v>20</v>
       </c>
     </row>
-    <row r="25" spans="1:18" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A25" s="11"/>
-      <c r="B25" s="10" t="s">
+    <row r="25" spans="1:18" ht="17.25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A25" s="10"/>
+      <c r="B25" s="9" t="s">
         <v>48</v>
       </c>
-      <c r="C25" s="12"/>
+      <c r="C25" s="11"/>
       <c r="D25" s="6"/>
       <c r="E25" s="6"/>
       <c r="F25" s="6"/>
@@ -2442,16 +2492,16 @@
       <c r="O25" s="7"/>
       <c r="P25" s="6"/>
       <c r="Q25" s="6"/>
-      <c r="R25" s="13"/>
-    </row>
-    <row r="26" spans="1:18" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A26" s="14" t="s">
+      <c r="R25" s="12"/>
+    </row>
+    <row r="26" spans="1:18" ht="17.25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A26" s="13" t="s">
         <v>49</v>
       </c>
-      <c r="B26" s="10" t="s">
+      <c r="B26" s="9" t="s">
         <v>50</v>
       </c>
-      <c r="C26" s="12" t="s">
+      <c r="C26" s="11" t="s">
         <v>70</v>
       </c>
       <c r="D26" s="7">
@@ -2487,7 +2537,7 @@
       <c r="N26" s="7">
         <v>1</v>
       </c>
-      <c r="O26" s="10" t="s">
+      <c r="O26" s="9" t="s">
         <v>21</v>
       </c>
       <c r="P26" s="7">
@@ -2496,16 +2546,16 @@
       <c r="Q26" s="7">
         <v>0</v>
       </c>
-      <c r="R26" s="10" t="s">
+      <c r="R26" s="9" t="s">
         <v>20</v>
       </c>
     </row>
-    <row r="27" spans="1:18" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A27" s="11"/>
-      <c r="B27" s="10" t="s">
+    <row r="27" spans="1:18" ht="17.25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A27" s="10"/>
+      <c r="B27" s="9" t="s">
         <v>51</v>
       </c>
-      <c r="C27" s="12"/>
+      <c r="C27" s="11"/>
       <c r="D27" s="6"/>
       <c r="E27" s="6"/>
       <c r="F27" s="6"/>
@@ -2520,16 +2570,16 @@
       <c r="O27" s="7"/>
       <c r="P27" s="6"/>
       <c r="Q27" s="6"/>
-      <c r="R27" s="13"/>
-    </row>
-    <row r="28" spans="1:18" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A28" s="14" t="s">
+      <c r="R27" s="12"/>
+    </row>
+    <row r="28" spans="1:18" ht="17.25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A28" s="13" t="s">
         <v>52</v>
       </c>
-      <c r="B28" s="10" t="s">
+      <c r="B28" s="9" t="s">
         <v>53</v>
       </c>
-      <c r="C28" s="12" t="s">
+      <c r="C28" s="11" t="s">
         <v>71</v>
       </c>
       <c r="D28" s="7">
@@ -2565,7 +2615,7 @@
       <c r="N28" s="7">
         <v>0</v>
       </c>
-      <c r="O28" s="10" t="s">
+      <c r="O28" s="9" t="s">
         <v>21</v>
       </c>
       <c r="P28" s="7">
@@ -2574,18 +2624,18 @@
       <c r="Q28" s="7">
         <v>0</v>
       </c>
-      <c r="R28" s="10" t="s">
+      <c r="R28" s="9" t="s">
         <v>54</v>
       </c>
     </row>
-    <row r="29" spans="1:18" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A29" s="14" t="s">
+    <row r="29" spans="1:18" ht="17.25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A29" s="13" t="s">
         <v>55</v>
       </c>
-      <c r="B29" s="10" t="s">
+      <c r="B29" s="9" t="s">
         <v>54</v>
       </c>
-      <c r="C29" s="12"/>
+      <c r="C29" s="11"/>
       <c r="D29" s="7">
         <v>0</v>
       </c>
@@ -2619,7 +2669,7 @@
       <c r="N29" s="7">
         <v>1</v>
       </c>
-      <c r="O29" s="10" t="s">
+      <c r="O29" s="9" t="s">
         <v>56</v>
       </c>
       <c r="P29" s="7">
@@ -2628,18 +2678,18 @@
       <c r="Q29" s="7">
         <v>0</v>
       </c>
-      <c r="R29" s="10" t="s">
+      <c r="R29" s="9" t="s">
         <v>20</v>
       </c>
     </row>
-    <row r="30" spans="1:18" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A30" s="14" t="s">
+    <row r="30" spans="1:18" ht="17.25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A30" s="13" t="s">
         <v>57</v>
       </c>
-      <c r="B30" s="10" t="s">
+      <c r="B30" s="9" t="s">
         <v>58</v>
       </c>
-      <c r="C30" s="12" t="s">
+      <c r="C30" s="11" t="s">
         <v>72</v>
       </c>
       <c r="D30" s="7">
@@ -2675,7 +2725,7 @@
       <c r="N30" s="7">
         <v>0</v>
       </c>
-      <c r="O30" s="10" t="s">
+      <c r="O30" s="9" t="s">
         <v>21</v>
       </c>
       <c r="P30" s="7">
@@ -2684,18 +2734,18 @@
       <c r="Q30" s="7">
         <v>0</v>
       </c>
-      <c r="R30" s="10" t="s">
+      <c r="R30" s="9" t="s">
         <v>59</v>
       </c>
     </row>
-    <row r="31" spans="1:18" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A31" s="14" t="s">
+    <row r="31" spans="1:18" ht="17.25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A31" s="13" t="s">
         <v>60</v>
       </c>
-      <c r="B31" s="10" t="s">
+      <c r="B31" s="9" t="s">
         <v>59</v>
       </c>
-      <c r="C31" s="12"/>
+      <c r="C31" s="11"/>
       <c r="D31" s="7">
         <v>0</v>
       </c>
@@ -2729,7 +2779,7 @@
       <c r="N31" s="7">
         <v>1</v>
       </c>
-      <c r="O31" s="10" t="s">
+      <c r="O31" s="9" t="s">
         <v>61</v>
       </c>
       <c r="P31" s="7">
@@ -2738,16 +2788,16 @@
       <c r="Q31" s="7">
         <v>0</v>
       </c>
-      <c r="R31" s="10" t="s">
+      <c r="R31" s="9" t="s">
         <v>20</v>
       </c>
     </row>
-    <row r="32" spans="1:18" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A32" s="11"/>
-      <c r="B32" s="10" t="s">
+    <row r="32" spans="1:18" ht="17.25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A32" s="10"/>
+      <c r="B32" s="9" t="s">
         <v>62</v>
       </c>
-      <c r="C32" s="12"/>
+      <c r="C32" s="11"/>
       <c r="D32" s="6"/>
       <c r="E32" s="6"/>
       <c r="F32" s="6"/>
@@ -2762,14 +2812,14 @@
       <c r="O32" s="7"/>
       <c r="P32" s="6"/>
       <c r="Q32" s="6"/>
-      <c r="R32" s="13"/>
-    </row>
-    <row r="33" spans="1:18" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A33" s="11"/>
-      <c r="B33" s="10" t="s">
+      <c r="R32" s="12"/>
+    </row>
+    <row r="33" spans="1:18" ht="17.25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A33" s="10"/>
+      <c r="B33" s="9" t="s">
         <v>63</v>
       </c>
-      <c r="C33" s="12"/>
+      <c r="C33" s="11"/>
       <c r="D33" s="6"/>
       <c r="E33" s="6"/>
       <c r="F33" s="6"/>
@@ -2784,16 +2834,16 @@
       <c r="O33" s="7"/>
       <c r="P33" s="6"/>
       <c r="Q33" s="6"/>
-      <c r="R33" s="13"/>
-    </row>
-    <row r="34" spans="1:18" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A34" s="14" t="s">
+      <c r="R33" s="12"/>
+    </row>
+    <row r="34" spans="1:18" ht="17.25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A34" s="13" t="s">
         <v>64</v>
       </c>
-      <c r="B34" s="10" t="s">
+      <c r="B34" s="9" t="s">
         <v>65</v>
       </c>
-      <c r="C34" s="12" t="s">
+      <c r="C34" s="11" t="s">
         <v>73</v>
       </c>
       <c r="D34" s="7">
@@ -2838,16 +2888,16 @@
       <c r="Q34" s="7">
         <v>0</v>
       </c>
-      <c r="R34" s="10" t="s">
+      <c r="R34" s="9" t="s">
         <v>26</v>
       </c>
     </row>
-    <row r="35" spans="1:18" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A35" s="11"/>
-      <c r="B35" s="10" t="s">
+    <row r="35" spans="1:18" ht="17.25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A35" s="10"/>
+      <c r="B35" s="9" t="s">
         <v>66</v>
       </c>
-      <c r="C35" s="12"/>
+      <c r="C35" s="11"/>
       <c r="D35" s="6"/>
       <c r="E35" s="6"/>
       <c r="F35" s="6"/>
@@ -2862,9 +2912,9 @@
       <c r="O35" s="6"/>
       <c r="P35" s="6"/>
       <c r="Q35" s="6"/>
-      <c r="R35" s="13"/>
-    </row>
-    <row r="36" spans="1:18" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="R35" s="12"/>
+    </row>
+    <row r="36" spans="1:18" ht="17.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B36" s="4"/>
     </row>
   </sheetData>

</xml_diff>